<commit_message>
chore(pmo-pert): remove deprecated Timeline/Resources helpers; regenerate template
- Delete scripts/helpers/wb_timeline.py and scripts/helpers/wb_resources.py
  along with their test modules. Both modules implemented sheets that the
  v2 refactor removed (Issue #1 — Resources held % presented as effort;
  Issue #4 — Timeline Gantt was sequential and misleading).
- Regenerate assets/pert-template.xlsx by running the v2 generator on the
  updated sample-input.json so the bundled reference template matches the
  4-sheet layout.
- Test suite is green (135 tests) and the structural CI test suite passes.
- End-to-end smoke: sample workbook opens with 4 sheets, Resource Plan
  totals are =SUM formulas over per-week PD numerics, Summary shows the
  Low/Medium/High bands plus Calendar Duration = 12 weeks.
</commit_message>
<xml_diff>
--- a/project-management/skills/pmo-pert-estimate/assets/pert-template.xlsx
+++ b/project-management/skills/pmo-pert-estimate/assets/pert-template.xlsx
@@ -8,10 +8,9 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="WBS" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Timeline" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resources" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risks" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resource Plan" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risks" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -20,10 +19,8 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="1">
-    <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
-  </numFmts>
-  <fonts count="8">
+  <numFmts count="0"/>
+  <fonts count="7">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -44,19 +41,14 @@
     </font>
     <font/>
     <font>
-      <b val="1"/>
-      <u val="single"/>
-    </font>
-    <font>
       <i val="1"/>
-      <sz val="9"/>
     </font>
     <font>
       <b val="1"/>
       <color rgb="FFFF0000"/>
     </font>
   </fonts>
-  <fills count="9">
+  <fills count="7">
     <fill>
       <patternFill/>
     </fill>
@@ -85,17 +77,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFF0000"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FF4472C4"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFA500"/>
+        <fgColor rgb="FFFFEB9C"/>
       </patternFill>
     </fill>
   </fills>
@@ -114,7 +96,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="29">
+  <cellXfs count="22">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -153,29 +135,16 @@
     <xf numFmtId="4" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="4" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="4" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="4" fontId="0" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -2087,557 +2056,404 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I34"/>
+  <dimension ref="A1:P6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="8" customWidth="1" min="1" max="1"/>
-    <col width="40" customWidth="1" min="2" max="2"/>
+    <col width="26" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
     <col width="14" customWidth="1" min="3" max="3"/>
-    <col width="12" customWidth="1" min="4" max="4"/>
-    <col width="6" customWidth="1" min="5" max="5"/>
-    <col width="6" customWidth="1" min="6" max="6"/>
-    <col width="6" customWidth="1" min="7" max="7"/>
-    <col width="6" customWidth="1" min="8" max="8"/>
-    <col width="6" customWidth="1" min="9" max="9"/>
+    <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="10" customWidth="1" min="5" max="5"/>
+    <col width="10" customWidth="1" min="6" max="6"/>
+    <col width="10" customWidth="1" min="7" max="7"/>
+    <col width="10" customWidth="1" min="8" max="8"/>
+    <col width="10" customWidth="1" min="9" max="9"/>
+    <col width="10" customWidth="1" min="10" max="10"/>
+    <col width="10" customWidth="1" min="11" max="11"/>
+    <col width="10" customWidth="1" min="12" max="12"/>
+    <col width="10" customWidth="1" min="13" max="13"/>
+    <col width="10" customWidth="1" min="14" max="14"/>
+    <col width="10" customWidth="1" min="15" max="15"/>
+    <col width="14" customWidth="1" min="16" max="16"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>ID</t>
+          <t>Role</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>Phase/WP/Activity</t>
+          <t>Code</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>PERT Duration</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>σ</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>P1</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>P2</t>
-        </is>
-      </c>
-      <c r="G1" s="1" t="inlineStr">
-        <is>
-          <t>P3</t>
-        </is>
-      </c>
-      <c r="H1" s="1" t="inlineStr">
-        <is>
-          <t>P4</t>
-        </is>
-      </c>
-      <c r="I1" s="1" t="inlineStr">
-        <is>
-          <t>P5</t>
+          <t>Type</t>
+        </is>
+      </c>
+      <c r="D1" s="14" t="inlineStr">
+        <is>
+          <t>W1</t>
+        </is>
+      </c>
+      <c r="E1" s="14" t="inlineStr">
+        <is>
+          <t>W2</t>
+        </is>
+      </c>
+      <c r="F1" s="14" t="inlineStr">
+        <is>
+          <t>W3</t>
+        </is>
+      </c>
+      <c r="G1" s="14" t="inlineStr">
+        <is>
+          <t>W4</t>
+        </is>
+      </c>
+      <c r="H1" s="14" t="inlineStr">
+        <is>
+          <t>W5</t>
+        </is>
+      </c>
+      <c r="I1" s="14" t="inlineStr">
+        <is>
+          <t>W6</t>
+        </is>
+      </c>
+      <c r="J1" s="14" t="inlineStr">
+        <is>
+          <t>W7</t>
+        </is>
+      </c>
+      <c r="K1" s="14" t="inlineStr">
+        <is>
+          <t>W8</t>
+        </is>
+      </c>
+      <c r="L1" s="14" t="inlineStr">
+        <is>
+          <t>W9</t>
+        </is>
+      </c>
+      <c r="M1" s="14" t="inlineStr">
+        <is>
+          <t>W10</t>
+        </is>
+      </c>
+      <c r="N1" s="14" t="inlineStr">
+        <is>
+          <t>W11</t>
+        </is>
+      </c>
+      <c r="O1" s="14" t="inlineStr">
+        <is>
+          <t>W12</t>
+        </is>
+      </c>
+      <c r="P1" s="1" t="inlineStr">
+        <is>
+          <t>TOTAL (PD)</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2">
-        <f>WBS!A2</f>
-        <v/>
-      </c>
-      <c r="B2">
-        <f>WBS!B2&amp;IF(WBS!C2&lt;&gt;"", " "&amp;WBS!C2, "")&amp;IF(WBS!D2&lt;&gt;"", " "&amp;WBS!D2, "")</f>
-        <v/>
-      </c>
-      <c r="C2">
-        <f>WBS!L2</f>
-        <v/>
-      </c>
-      <c r="D2">
-        <f>WBS!M2</f>
-        <v/>
+      <c r="C2" s="15" t="inlineStr">
+        <is>
+          <t>Week of</t>
+        </is>
+      </c>
+      <c r="D2" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-06</t>
+        </is>
+      </c>
+      <c r="E2" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-13</t>
+        </is>
+      </c>
+      <c r="F2" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-20</t>
+        </is>
+      </c>
+      <c r="G2" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-27</t>
+        </is>
+      </c>
+      <c r="H2" s="15" t="inlineStr">
+        <is>
+          <t>2026-05-04</t>
+        </is>
+      </c>
+      <c r="I2" s="15" t="inlineStr">
+        <is>
+          <t>2026-05-11</t>
+        </is>
+      </c>
+      <c r="J2" s="15" t="inlineStr">
+        <is>
+          <t>2026-05-18</t>
+        </is>
+      </c>
+      <c r="K2" s="15" t="inlineStr">
+        <is>
+          <t>2026-05-25</t>
+        </is>
+      </c>
+      <c r="L2" s="15" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="M2" s="15" t="inlineStr">
+        <is>
+          <t>2026-06-08</t>
+        </is>
+      </c>
+      <c r="N2" s="15" t="inlineStr">
+        <is>
+          <t>2026-06-15</t>
+        </is>
+      </c>
+      <c r="O2" s="15" t="inlineStr">
+        <is>
+          <t>2026-06-22</t>
+        </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3">
-        <f>WBS!A3</f>
-        <v/>
-      </c>
-      <c r="B3">
-        <f>WBS!B3&amp;IF(WBS!C3&lt;&gt;"", " "&amp;WBS!C3, "")&amp;IF(WBS!D3&lt;&gt;"", " "&amp;WBS!D3, "")</f>
-        <v/>
-      </c>
-      <c r="C3">
-        <f>WBS!L3</f>
-        <v/>
-      </c>
-      <c r="D3">
-        <f>WBS!M3</f>
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Project Manager</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>PM</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>billable</t>
+        </is>
+      </c>
+      <c r="D3" s="16" t="n">
+        <v>3.58</v>
+      </c>
+      <c r="E3" s="16" t="n">
+        <v>3.58</v>
+      </c>
+      <c r="F3" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="G3" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="H3" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="I3" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="J3" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="K3" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="L3" s="16" t="n">
+        <v>0.83</v>
+      </c>
+      <c r="M3" s="16" t="n">
+        <v>0.83</v>
+      </c>
+      <c r="N3" s="16" t="n">
+        <v>0.83</v>
+      </c>
+      <c r="O3" s="16" t="n">
+        <v>0.83</v>
+      </c>
+      <c r="P3" s="17">
+        <f>SUM(D3:O3)</f>
         <v/>
       </c>
     </row>
     <row r="4">
-      <c r="A4">
-        <f>WBS!A4</f>
-        <v/>
-      </c>
-      <c r="B4">
-        <f>WBS!B4&amp;IF(WBS!C4&lt;&gt;"", " "&amp;WBS!C4, "")&amp;IF(WBS!D4&lt;&gt;"", " "&amp;WBS!D4, "")</f>
-        <v/>
-      </c>
-      <c r="C4">
-        <f>WBS!L4</f>
-        <v/>
-      </c>
-      <c r="D4">
-        <f>WBS!M4</f>
-        <v/>
-      </c>
-      <c r="E4" s="14" t="n"/>
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>QA Engineer</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>QA</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>billable</t>
+        </is>
+      </c>
+      <c r="D4" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="E4" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="F4" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="G4" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="H4" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="I4" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="J4" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="K4" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="L4" s="16" t="n">
+        <v>2.38</v>
+      </c>
+      <c r="M4" s="16" t="n">
+        <v>2.38</v>
+      </c>
+      <c r="N4" s="16" t="n">
+        <v>2.38</v>
+      </c>
+      <c r="O4" s="16" t="n">
+        <v>2.38</v>
+      </c>
+      <c r="P4" s="17">
+        <f>SUM(D4:O4)</f>
+        <v/>
+      </c>
     </row>
     <row r="5">
-      <c r="A5">
-        <f>WBS!A5</f>
-        <v/>
-      </c>
-      <c r="B5">
-        <f>WBS!B5&amp;IF(WBS!C5&lt;&gt;"", " "&amp;WBS!C5, "")&amp;IF(WBS!D5&lt;&gt;"", " "&amp;WBS!D5, "")</f>
-        <v/>
-      </c>
-      <c r="C5">
-        <f>WBS!L5</f>
-        <v/>
-      </c>
-      <c r="D5">
-        <f>WBS!M5</f>
-        <v/>
-      </c>
-      <c r="E5" s="14" t="n"/>
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Senior Developer</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>SD</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>billable</t>
+        </is>
+      </c>
+      <c r="D5" s="16" t="n">
+        <v>3.17</v>
+      </c>
+      <c r="E5" s="16" t="n">
+        <v>3.17</v>
+      </c>
+      <c r="F5" s="16" t="n">
+        <v>4.12</v>
+      </c>
+      <c r="G5" s="16" t="n">
+        <v>4.12</v>
+      </c>
+      <c r="H5" s="16" t="n">
+        <v>4.12</v>
+      </c>
+      <c r="I5" s="16" t="n">
+        <v>4.12</v>
+      </c>
+      <c r="J5" s="16" t="n">
+        <v>4.12</v>
+      </c>
+      <c r="K5" s="16" t="n">
+        <v>4.12</v>
+      </c>
+      <c r="L5" s="18" t="n">
+        <v>4.66</v>
+      </c>
+      <c r="M5" s="16" t="n">
+        <v>0.54</v>
+      </c>
+      <c r="N5" s="16" t="n">
+        <v>0.54</v>
+      </c>
+      <c r="O5" s="16" t="n">
+        <v>0.54</v>
+      </c>
+      <c r="P5" s="17">
+        <f>SUM(D5:O5)</f>
+        <v/>
+      </c>
     </row>
     <row r="6">
-      <c r="A6">
-        <f>WBS!A6</f>
-        <v/>
-      </c>
-      <c r="B6">
-        <f>WBS!B6&amp;IF(WBS!C6&lt;&gt;"", " "&amp;WBS!C6, "")&amp;IF(WBS!D6&lt;&gt;"", " "&amp;WBS!D6, "")</f>
-        <v/>
-      </c>
-      <c r="C6">
-        <f>WBS!L6</f>
-        <v/>
-      </c>
-      <c r="D6">
-        <f>WBS!M6</f>
-        <v/>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7">
-        <f>WBS!A7</f>
-        <v/>
-      </c>
-      <c r="B7">
-        <f>WBS!B7&amp;IF(WBS!C7&lt;&gt;"", " "&amp;WBS!C7, "")&amp;IF(WBS!D7&lt;&gt;"", " "&amp;WBS!D7, "")</f>
-        <v/>
-      </c>
-      <c r="C7">
-        <f>WBS!L7</f>
-        <v/>
-      </c>
-      <c r="D7">
-        <f>WBS!M7</f>
-        <v/>
-      </c>
-      <c r="E7" s="15" t="n"/>
-    </row>
-    <row r="8">
-      <c r="A8">
-        <f>WBS!A8</f>
-        <v/>
-      </c>
-      <c r="B8">
-        <f>WBS!B8&amp;IF(WBS!C8&lt;&gt;"", " "&amp;WBS!C8, "")&amp;IF(WBS!D8&lt;&gt;"", " "&amp;WBS!D8, "")</f>
-        <v/>
-      </c>
-      <c r="C8">
-        <f>WBS!L8</f>
-        <v/>
-      </c>
-      <c r="D8">
-        <f>WBS!M8</f>
-        <v/>
-      </c>
-      <c r="E8" s="15" t="n"/>
-      <c r="F8" s="15" t="n"/>
-    </row>
-    <row r="9">
-      <c r="A9">
-        <f>WBS!A9</f>
-        <v/>
-      </c>
-      <c r="B9">
-        <f>WBS!B9&amp;IF(WBS!C9&lt;&gt;"", " "&amp;WBS!C9, "")&amp;IF(WBS!D9&lt;&gt;"", " "&amp;WBS!D9, "")</f>
-        <v/>
-      </c>
-      <c r="C9">
-        <f>WBS!L9</f>
-        <v/>
-      </c>
-      <c r="D9">
-        <f>WBS!M9</f>
-        <v/>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10">
-        <f>WBS!A10</f>
-        <v/>
-      </c>
-      <c r="B10">
-        <f>WBS!B10&amp;IF(WBS!C10&lt;&gt;"", " "&amp;WBS!C10, "")&amp;IF(WBS!D10&lt;&gt;"", " "&amp;WBS!D10, "")</f>
-        <v/>
-      </c>
-      <c r="C10">
-        <f>WBS!L10</f>
-        <v/>
-      </c>
-      <c r="D10">
-        <f>WBS!M10</f>
-        <v/>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11">
-        <f>WBS!A11</f>
-        <v/>
-      </c>
-      <c r="B11">
-        <f>WBS!B11&amp;IF(WBS!C11&lt;&gt;"", " "&amp;WBS!C11, "")&amp;IF(WBS!D11&lt;&gt;"", " "&amp;WBS!D11, "")</f>
-        <v/>
-      </c>
-      <c r="C11">
-        <f>WBS!L11</f>
-        <v/>
-      </c>
-      <c r="D11">
-        <f>WBS!M11</f>
-        <v/>
-      </c>
-      <c r="E11" s="14" t="n"/>
-      <c r="F11" s="14" t="n"/>
-    </row>
-    <row r="12">
-      <c r="A12">
-        <f>WBS!A12</f>
-        <v/>
-      </c>
-      <c r="B12">
-        <f>WBS!B12&amp;IF(WBS!C12&lt;&gt;"", " "&amp;WBS!C12, "")&amp;IF(WBS!D12&lt;&gt;"", " "&amp;WBS!D12, "")</f>
-        <v/>
-      </c>
-      <c r="C12">
-        <f>WBS!L12</f>
-        <v/>
-      </c>
-      <c r="D12">
-        <f>WBS!M12</f>
-        <v/>
-      </c>
-      <c r="F12" s="14" t="n"/>
-    </row>
-    <row r="13">
-      <c r="A13">
-        <f>WBS!A13</f>
-        <v/>
-      </c>
-      <c r="B13">
-        <f>WBS!B13&amp;IF(WBS!C13&lt;&gt;"", " "&amp;WBS!C13, "")&amp;IF(WBS!D13&lt;&gt;"", " "&amp;WBS!D13, "")</f>
-        <v/>
-      </c>
-      <c r="C13">
-        <f>WBS!L13</f>
-        <v/>
-      </c>
-      <c r="D13">
-        <f>WBS!M13</f>
-        <v/>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14">
-        <f>WBS!A14</f>
-        <v/>
-      </c>
-      <c r="B14">
-        <f>WBS!B14&amp;IF(WBS!C14&lt;&gt;"", " "&amp;WBS!C14, "")&amp;IF(WBS!D14&lt;&gt;"", " "&amp;WBS!D14, "")</f>
-        <v/>
-      </c>
-      <c r="C14">
-        <f>WBS!L14</f>
-        <v/>
-      </c>
-      <c r="D14">
-        <f>WBS!M14</f>
-        <v/>
-      </c>
-      <c r="F14" s="14" t="n"/>
-      <c r="G14" s="14" t="n"/>
-    </row>
-    <row r="15">
-      <c r="A15">
-        <f>WBS!A15</f>
-        <v/>
-      </c>
-      <c r="B15">
-        <f>WBS!B15&amp;IF(WBS!C15&lt;&gt;"", " "&amp;WBS!C15, "")&amp;IF(WBS!D15&lt;&gt;"", " "&amp;WBS!D15, "")</f>
-        <v/>
-      </c>
-      <c r="C15">
-        <f>WBS!L15</f>
-        <v/>
-      </c>
-      <c r="D15">
-        <f>WBS!M15</f>
-        <v/>
-      </c>
-      <c r="F15" s="15" t="n"/>
-      <c r="G15" s="15" t="n"/>
-    </row>
-    <row r="16">
-      <c r="A16">
-        <f>WBS!A16</f>
-        <v/>
-      </c>
-      <c r="B16">
-        <f>WBS!B16&amp;IF(WBS!C16&lt;&gt;"", " "&amp;WBS!C16, "")&amp;IF(WBS!D16&lt;&gt;"", " "&amp;WBS!D16, "")</f>
-        <v/>
-      </c>
-      <c r="C16">
-        <f>WBS!L16</f>
-        <v/>
-      </c>
-      <c r="D16">
-        <f>WBS!M16</f>
-        <v/>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17">
-        <f>WBS!A17</f>
-        <v/>
-      </c>
-      <c r="B17">
-        <f>WBS!B17&amp;IF(WBS!C17&lt;&gt;"", " "&amp;WBS!C17, "")&amp;IF(WBS!D17&lt;&gt;"", " "&amp;WBS!D17, "")</f>
-        <v/>
-      </c>
-      <c r="C17">
-        <f>WBS!L17</f>
-        <v/>
-      </c>
-      <c r="D17">
-        <f>WBS!M17</f>
-        <v/>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18">
-        <f>WBS!A18</f>
-        <v/>
-      </c>
-      <c r="B18">
-        <f>WBS!B18&amp;IF(WBS!C18&lt;&gt;"", " "&amp;WBS!C18, "")&amp;IF(WBS!D18&lt;&gt;"", " "&amp;WBS!D18, "")</f>
-        <v/>
-      </c>
-      <c r="C18">
-        <f>WBS!L18</f>
-        <v/>
-      </c>
-      <c r="D18">
-        <f>WBS!M18</f>
-        <v/>
-      </c>
-      <c r="G18" s="14" t="n"/>
-      <c r="H18" s="14" t="n"/>
-    </row>
-    <row r="19">
-      <c r="A19">
-        <f>WBS!A19</f>
-        <v/>
-      </c>
-      <c r="B19">
-        <f>WBS!B19&amp;IF(WBS!C19&lt;&gt;"", " "&amp;WBS!C19, "")&amp;IF(WBS!D19&lt;&gt;"", " "&amp;WBS!D19, "")</f>
-        <v/>
-      </c>
-      <c r="C19">
-        <f>WBS!L19</f>
-        <v/>
-      </c>
-      <c r="D19">
-        <f>WBS!M19</f>
-        <v/>
-      </c>
-      <c r="H19" s="14" t="n"/>
-    </row>
-    <row r="20">
-      <c r="A20">
-        <f>WBS!A20</f>
-        <v/>
-      </c>
-      <c r="B20">
-        <f>WBS!B20&amp;IF(WBS!C20&lt;&gt;"", " "&amp;WBS!C20, "")&amp;IF(WBS!D20&lt;&gt;"", " "&amp;WBS!D20, "")</f>
-        <v/>
-      </c>
-      <c r="C20">
-        <f>WBS!L20</f>
-        <v/>
-      </c>
-      <c r="D20">
-        <f>WBS!M20</f>
-        <v/>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21">
-        <f>WBS!A21</f>
-        <v/>
-      </c>
-      <c r="B21">
-        <f>WBS!B21&amp;IF(WBS!C21&lt;&gt;"", " "&amp;WBS!C21, "")&amp;IF(WBS!D21&lt;&gt;"", " "&amp;WBS!D21, "")</f>
-        <v/>
-      </c>
-      <c r="C21">
-        <f>WBS!L21</f>
-        <v/>
-      </c>
-      <c r="D21">
-        <f>WBS!M21</f>
-        <v/>
-      </c>
-      <c r="H21" s="14" t="n"/>
-      <c r="I21" s="14" t="n"/>
-    </row>
-    <row r="22">
-      <c r="A22">
-        <f>WBS!A22</f>
-        <v/>
-      </c>
-      <c r="B22">
-        <f>WBS!B22&amp;IF(WBS!C22&lt;&gt;"", " "&amp;WBS!C22, "")&amp;IF(WBS!D22&lt;&gt;"", " "&amp;WBS!D22, "")</f>
-        <v/>
-      </c>
-      <c r="C22">
-        <f>WBS!L22</f>
-        <v/>
-      </c>
-      <c r="D22">
-        <f>WBS!M22</f>
-        <v/>
-      </c>
-      <c r="I22" s="14" t="n"/>
-    </row>
-    <row r="24">
-      <c r="A24" s="16" t="inlineStr">
-        <is>
-          <t>Critical Path</t>
-        </is>
-      </c>
-      <c r="B24" t="inlineStr">
-        <is>
-          <t>1.1.1 → 1.1.2 → 2.1.1 → 2.1.2 → 2.2.1 → 3.1.1 → 3.1.2 → 3.2.1 → 3.2.2</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="16" t="inlineStr">
-        <is>
-          <t>Total PERT Duration</t>
-        </is>
-      </c>
-      <c r="B25">
-        <f>WBS!L23</f>
-        <v/>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="16" t="inlineStr">
-        <is>
-          <t>CI 68%</t>
-        </is>
-      </c>
-      <c r="B26">
-        <f>WBS!L23&amp;" ± "&amp;WBS!M23</f>
-        <v/>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="16" t="inlineStr">
-        <is>
-          <t>CI 95%</t>
-        </is>
-      </c>
-      <c r="B27">
-        <f>WBS!L23&amp;" ± 2×"&amp;WBS!M23</f>
-        <v/>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" s="16" t="inlineStr">
-        <is>
-          <t>Start Date</t>
-        </is>
-      </c>
-      <c r="B28" s="17" t="n">
-        <v>46118</v>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" s="16" t="inlineStr">
-        <is>
-          <t>End Date</t>
-        </is>
-      </c>
-      <c r="B29" s="17" t="n">
-        <v>46178</v>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" s="18" t="inlineStr">
-        <is>
-          <t>Legend</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" s="14" t="inlineStr"/>
-      <c r="B32" t="inlineStr">
-        <is>
-          <t>Critical Path</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" s="15" t="inlineStr"/>
-      <c r="B33" t="inlineStr">
-        <is>
-          <t>Parallel Activity</t>
-        </is>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" s="19" t="inlineStr"/>
-      <c r="B34" t="inlineStr">
-        <is>
-          <t>Continuous Activity</t>
-        </is>
+      <c r="A6" s="11" t="inlineStr">
+        <is>
+          <t>Weekly TOTAL</t>
+        </is>
+      </c>
+      <c r="D6" s="12">
+        <f>SUM(D3:D5)</f>
+        <v/>
+      </c>
+      <c r="E6" s="12">
+        <f>SUM(E3:E5)</f>
+        <v/>
+      </c>
+      <c r="F6" s="12">
+        <f>SUM(F3:F5)</f>
+        <v/>
+      </c>
+      <c r="G6" s="12">
+        <f>SUM(G3:G5)</f>
+        <v/>
+      </c>
+      <c r="H6" s="12">
+        <f>SUM(H3:H5)</f>
+        <v/>
+      </c>
+      <c r="I6" s="12">
+        <f>SUM(I3:I5)</f>
+        <v/>
+      </c>
+      <c r="J6" s="12">
+        <f>SUM(J3:J5)</f>
+        <v/>
+      </c>
+      <c r="K6" s="12">
+        <f>SUM(K3:K5)</f>
+        <v/>
+      </c>
+      <c r="L6" s="12">
+        <f>SUM(L3:L5)</f>
+        <v/>
+      </c>
+      <c r="M6" s="12">
+        <f>SUM(M3:M5)</f>
+        <v/>
+      </c>
+      <c r="N6" s="12">
+        <f>SUM(N3:N5)</f>
+        <v/>
+      </c>
+      <c r="O6" s="12">
+        <f>SUM(O3:O5)</f>
+        <v/>
+      </c>
+      <c r="P6" s="12">
+        <f>SUM(D6:O6)</f>
+        <v/>
       </c>
     </row>
   </sheetData>
@@ -2646,358 +2462,6 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:H12"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="D1" s="20" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="E1" s="20" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="F1" s="20" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="21" t="inlineStr">
-        <is>
-          <t>Phase</t>
-        </is>
-      </c>
-      <c r="B2" s="21" t="inlineStr">
-        <is>
-          <t>Description</t>
-        </is>
-      </c>
-      <c r="C2" s="21" t="inlineStr">
-        <is>
-          <t>Team</t>
-        </is>
-      </c>
-      <c r="D2" s="22" t="inlineStr">
-        <is>
-          <t>Project Manager</t>
-        </is>
-      </c>
-      <c r="E2" s="22" t="inlineStr">
-        <is>
-          <t>Senior Developer</t>
-        </is>
-      </c>
-      <c r="F2" s="22" t="inlineStr">
-        <is>
-          <t>QA Engineer</t>
-        </is>
-      </c>
-      <c r="G2" s="22" t="inlineStr">
-        <is>
-          <t>TOTAL EFFORT</t>
-        </is>
-      </c>
-      <c r="H2" s="22" t="inlineStr">
-        <is>
-          <t>BILLABLE EFFORT</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="8" t="inlineStr">
-        <is>
-          <t>Analysis</t>
-        </is>
-      </c>
-      <c r="B3" s="8" t="inlineStr">
-        <is>
-          <t>Requirements analysis and planning</t>
-        </is>
-      </c>
-      <c r="C3" s="8" t="inlineStr">
-        <is>
-          <t>Management</t>
-        </is>
-      </c>
-      <c r="D3" s="23" t="n">
-        <v>8</v>
-      </c>
-      <c r="G3" s="24">
-        <f>SUM(D3:F3)</f>
-        <v/>
-      </c>
-      <c r="H3" s="24">
-        <f>SUMPRODUCT(D3:F3,(D$1:F$1="Y")*1)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="8" t="inlineStr">
-        <is>
-          <t>Design &amp; Development</t>
-        </is>
-      </c>
-      <c r="B4" s="8" t="inlineStr">
-        <is>
-          <t>System design and implementation</t>
-        </is>
-      </c>
-      <c r="C4" s="8" t="inlineStr">
-        <is>
-          <t>Management</t>
-        </is>
-      </c>
-      <c r="D4" s="23" t="n">
-        <v>5</v>
-      </c>
-      <c r="G4" s="24">
-        <f>SUM(D4:F4)</f>
-        <v/>
-      </c>
-      <c r="H4" s="24">
-        <f>SUMPRODUCT(D4:F4,(D$1:F$1="Y")*1)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="8" t="inlineStr">
-        <is>
-          <t>Testing &amp; Deployment</t>
-        </is>
-      </c>
-      <c r="B5" s="8" t="inlineStr">
-        <is>
-          <t>Quality assurance and production rollout</t>
-        </is>
-      </c>
-      <c r="C5" s="8" t="inlineStr">
-        <is>
-          <t>Management</t>
-        </is>
-      </c>
-      <c r="D5" s="23" t="n">
-        <v>5</v>
-      </c>
-      <c r="G5" s="24">
-        <f>SUM(D5:F5)</f>
-        <v/>
-      </c>
-      <c r="H5" s="24">
-        <f>SUMPRODUCT(D5:F5,(D$1:F$1="Y")*1)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="5" t="inlineStr">
-        <is>
-          <t>Subtotal — Management</t>
-        </is>
-      </c>
-      <c r="B6" s="5" t="inlineStr"/>
-      <c r="C6" s="5" t="inlineStr">
-        <is>
-          <t>Management</t>
-        </is>
-      </c>
-      <c r="D6" s="25">
-        <f>SUM(D3,D4,D5)</f>
-        <v/>
-      </c>
-      <c r="E6" s="25">
-        <f>SUM(E3,E4,E5)</f>
-        <v/>
-      </c>
-      <c r="F6" s="25">
-        <f>SUM(F3,F4,F5)</f>
-        <v/>
-      </c>
-      <c r="G6" s="26">
-        <f>SUM(D6:F6)</f>
-        <v/>
-      </c>
-      <c r="H6" s="26">
-        <f>SUMPRODUCT(D6:F6,(D$1:F$1="Y")*1)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="8" t="inlineStr">
-        <is>
-          <t>Analysis</t>
-        </is>
-      </c>
-      <c r="B7" s="8" t="inlineStr">
-        <is>
-          <t>Requirements analysis and planning</t>
-        </is>
-      </c>
-      <c r="C7" s="8" t="inlineStr">
-        <is>
-          <t>Development</t>
-        </is>
-      </c>
-      <c r="E7" s="23" t="n">
-        <v>13</v>
-      </c>
-      <c r="G7" s="24">
-        <f>SUM(D7:F7)</f>
-        <v/>
-      </c>
-      <c r="H7" s="24">
-        <f>SUMPRODUCT(D7:F7,(D$1:F$1="Y")*1)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="8" t="inlineStr">
-        <is>
-          <t>Design &amp; Development</t>
-        </is>
-      </c>
-      <c r="B8" s="8" t="inlineStr">
-        <is>
-          <t>System design and implementation</t>
-        </is>
-      </c>
-      <c r="C8" s="8" t="inlineStr">
-        <is>
-          <t>Development</t>
-        </is>
-      </c>
-      <c r="E8" s="23" t="n">
-        <v>28</v>
-      </c>
-      <c r="G8" s="24">
-        <f>SUM(D8:F8)</f>
-        <v/>
-      </c>
-      <c r="H8" s="24">
-        <f>SUMPRODUCT(D8:F8,(D$1:F$1="Y")*1)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="8" t="inlineStr">
-        <is>
-          <t>Testing &amp; Deployment</t>
-        </is>
-      </c>
-      <c r="B9" s="8" t="inlineStr">
-        <is>
-          <t>Quality assurance and production rollout</t>
-        </is>
-      </c>
-      <c r="C9" s="8" t="inlineStr">
-        <is>
-          <t>Development</t>
-        </is>
-      </c>
-      <c r="E9" s="23" t="n">
-        <v>9</v>
-      </c>
-      <c r="G9" s="24">
-        <f>SUM(D9:F9)</f>
-        <v/>
-      </c>
-      <c r="H9" s="24">
-        <f>SUMPRODUCT(D9:F9,(D$1:F$1="Y")*1)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="8" t="inlineStr">
-        <is>
-          <t>Testing &amp; Deployment</t>
-        </is>
-      </c>
-      <c r="B10" s="8" t="inlineStr">
-        <is>
-          <t>Quality assurance and production rollout</t>
-        </is>
-      </c>
-      <c r="C10" s="8" t="inlineStr">
-        <is>
-          <t>Development</t>
-        </is>
-      </c>
-      <c r="F10" s="23" t="n">
-        <v>12</v>
-      </c>
-      <c r="G10" s="24">
-        <f>SUM(D10:F10)</f>
-        <v/>
-      </c>
-      <c r="H10" s="24">
-        <f>SUMPRODUCT(D10:F10,(D$1:F$1="Y")*1)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="5" t="inlineStr">
-        <is>
-          <t>Subtotal — Development</t>
-        </is>
-      </c>
-      <c r="B11" s="5" t="inlineStr"/>
-      <c r="C11" s="5" t="inlineStr">
-        <is>
-          <t>Development</t>
-        </is>
-      </c>
-      <c r="D11" s="25">
-        <f>SUM(D7,D8,D9,D10)</f>
-        <v/>
-      </c>
-      <c r="E11" s="25">
-        <f>SUM(E7,E8,E9,E10)</f>
-        <v/>
-      </c>
-      <c r="F11" s="25">
-        <f>SUM(F7,F8,F9,F10)</f>
-        <v/>
-      </c>
-      <c r="G11" s="26">
-        <f>SUM(D11:F11)</f>
-        <v/>
-      </c>
-      <c r="H11" s="26">
-        <f>SUMPRODUCT(D11:F11,(D$1:F$1="Y")*1)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="11" t="inlineStr">
-        <is>
-          <t>TOTAL</t>
-        </is>
-      </c>
-      <c r="B12" s="11" t="inlineStr"/>
-      <c r="C12" s="11" t="inlineStr"/>
-      <c r="G12" s="27">
-        <f>SUM(G3:G11)</f>
-        <v/>
-      </c>
-      <c r="H12" s="27">
-        <f>SUM(H3:H11)</f>
-        <v/>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -3263,59 +2727,59 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="28" t="inlineStr">
+      <c r="A5" s="19" t="inlineStr">
         <is>
           <t>R4</t>
         </is>
       </c>
-      <c r="B5" s="28" t="inlineStr">
+      <c r="B5" s="19" t="inlineStr">
         <is>
           <t>UAT delayed due to client availability or environment issues</t>
         </is>
       </c>
-      <c r="C5" s="28" t="inlineStr">
+      <c r="C5" s="19" t="inlineStr">
         <is>
           <t>External</t>
         </is>
       </c>
-      <c r="D5" s="28" t="inlineStr">
+      <c r="D5" s="19" t="inlineStr">
         <is>
           <t>3</t>
         </is>
       </c>
-      <c r="E5" s="28" t="n">
+      <c r="E5" s="19" t="n">
         <v>4</v>
       </c>
-      <c r="F5" s="28" t="n">
+      <c r="F5" s="19" t="n">
         <v>4</v>
       </c>
-      <c r="G5" s="28">
+      <c r="G5" s="19">
         <f>E5*F5</f>
         <v/>
       </c>
-      <c r="H5" s="28">
+      <c r="H5" s="19">
         <f>IF(G5&gt;=15,"CRITICAL",IF(G5&gt;=10,"HIGH",IF(G5&gt;=5,"MEDIUM","LOW")))</f>
         <v/>
       </c>
-      <c r="I5" s="28" t="inlineStr">
+      <c r="I5" s="19" t="inlineStr">
         <is>
           <t>Mitigate</t>
         </is>
       </c>
-      <c r="J5" s="28" t="inlineStr">
+      <c r="J5" s="19" t="inlineStr">
         <is>
           <t>Agree on UAT schedule and environment setup checklist upfront</t>
         </is>
       </c>
-      <c r="K5" s="28" t="inlineStr">
+      <c r="K5" s="19" t="inlineStr">
         <is>
           <t>PM</t>
         </is>
       </c>
-      <c r="L5" s="28" t="n">
+      <c r="L5" s="19" t="n">
         <v>6</v>
       </c>
-      <c r="M5" s="28">
+      <c r="M5" s="19">
         <f>L5*500</f>
         <v/>
       </c>
@@ -3342,11 +2806,11 @@
         </is>
       </c>
       <c r="L8">
-        <f>L7*0.1</f>
+        <f>(WBS!H23*(1+0.1+0.05)+L7)*0.1</f>
         <v/>
       </c>
       <c r="M8">
-        <f>M7*0.1</f>
+        <f>(WBS!H23*(1+0.1+0.05)+L7)*0.1*500</f>
         <v/>
       </c>
     </row>
@@ -3355,17 +2819,17 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K21"/>
+  <dimension ref="A1:K28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="30" customWidth="1" min="1" max="1"/>
-    <col width="35" customWidth="1" min="2" max="2"/>
+    <col width="32" customWidth="1" min="1" max="1"/>
+    <col width="36" customWidth="1" min="2" max="2"/>
     <col width="14" customWidth="1" min="3" max="3"/>
     <col width="14" customWidth="1" min="4" max="4"/>
     <col width="14" customWidth="1" min="5" max="5"/>
@@ -3622,7 +3086,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Total PERT Effort (pd)</t>
+          <t>Tech PERT Effort (PD)</t>
         </is>
       </c>
       <c r="B7">
@@ -3633,140 +3097,176 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Total Billable Effort (pd)</t>
+          <t>PM Overhead (+10%) (PD)</t>
         </is>
       </c>
       <c r="B8">
-        <f>WBS!S23</f>
+        <f>B7*0.1</f>
         <v/>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Billable Ratio</t>
+          <t>DevOps Overhead (+5%) (PD)</t>
         </is>
       </c>
       <c r="B9">
-        <f>B8/B7</f>
+        <f>B7*0.05</f>
         <v/>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>σ Total Duration</t>
+          <t>Subtotal Tech + Overhead (PD)</t>
         </is>
       </c>
       <c r="B10">
-        <f>SQRT(SUMPRODUCT(K2:K4,K2:K4))</f>
+        <f>B7+B8+B9</f>
         <v/>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>CI 68% Lower</t>
+          <t>Contingency per-risk (PD)</t>
         </is>
       </c>
       <c r="B11">
-        <f>J5-B10</f>
+        <f>Risks!L7</f>
         <v/>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>CI 68% Upper</t>
+          <t>Low Band</t>
         </is>
       </c>
       <c r="B12">
-        <f>J5+B10</f>
+        <f>B10+B11</f>
         <v/>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>CI 95% Lower</t>
+          <t>Management Reserve (10%) (PD)</t>
         </is>
       </c>
       <c r="B13">
-        <f>J5-2*B10</f>
+        <f>B12*0.1</f>
         <v/>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>CI 95% Upper</t>
+          <t>Medium Band (recommended)</t>
         </is>
       </c>
       <c r="B14">
-        <f>J5+2*B10</f>
+        <f>B12+B13</f>
         <v/>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Total Contingency</t>
+          <t>High Band</t>
         </is>
       </c>
       <c r="B15">
-        <f>Risks!L7</f>
+        <f>B14*(1+0.12)</f>
         <v/>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Management Reserve</t>
+          <t>Total Billable Effort (PD)</t>
         </is>
       </c>
       <c r="B16">
-        <f>Risks!L8</f>
+        <f>WBS!S23</f>
         <v/>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Adjusted PERT Effort (pd)</t>
+          <t>Billable Ratio</t>
         </is>
       </c>
       <c r="B17">
-        <f>B7+B15+B16</f>
+        <f>B16/B7</f>
         <v/>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="16" t="inlineStr">
-        <is>
-          <t>Effort by Team</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Calendar Duration (weeks)</t>
+        </is>
+      </c>
+      <c r="B19" s="20" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="21" t="inlineStr">
+        <is>
+          <t>Effort by Team (PD)</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Development</t>
+        </is>
+      </c>
+      <c r="B22" s="16" t="n">
+        <v>46.83333333333333</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
         <is>
           <t>Management</t>
         </is>
       </c>
-      <c r="B20">
-        <f>Resources!G6</f>
-        <v/>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>Development</t>
-        </is>
-      </c>
-      <c r="B21">
-        <f>Resources!G11</f>
-        <v/>
+      <c r="B23" s="16" t="n">
+        <v>10.5</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="21" t="inlineStr">
+        <is>
+          <t>Sensitivity Scenarios</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Optimistic: 75 PD if stakeholder availability is high and no requirement changes occur</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Realistic: 92 PD (Fascia MEDIA) with current overhead and MR assumptions</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Pessimistic: 110 PD if external API integration delays force rework</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>